<commit_message>
Changed name to radio panel, to make room for the next sketch.
</commit_message>
<xml_diff>
--- a/Button tables.xlsx
+++ b/Button tables.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\cockpit_arduino\cockpit_joystick\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\cockpit_arduino\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2800FEED-7FD0-4079-BA5A-42FE48F57CEB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58493AB-5991-4EBB-BF6C-078A1D3566E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="8580" yWindow="3336" windowWidth="30420" windowHeight="18336" xr2:uid="{B42DDCD9-64C5-4A29-BEC7-73E9BF8FAFC9}"/>
+    <workbookView xWindow="60450" yWindow="12945" windowWidth="30420" windowHeight="18330" xr2:uid="{B42DDCD9-64C5-4A29-BEC7-73E9BF8FAFC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Radio Arduino" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="202" uniqueCount="113">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="119">
   <si>
     <t>Key</t>
   </si>
@@ -376,6 +376,24 @@
   </si>
   <si>
     <t>Vi gör en översättningstabell från signaler till knappar. I denna reserverar vi plats för knappar som definieras av kombinationer av signaler. Efter översättningen gör vi en manuell kod som löser dessa kombinationer.</t>
+  </si>
+  <si>
+    <t>Left Rotary CW</t>
+  </si>
+  <si>
+    <t>Left Rotary CCW</t>
+  </si>
+  <si>
+    <t>Right Rotary CW</t>
+  </si>
+  <si>
+    <t>Right Rotary CCW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CLR </t>
+  </si>
+  <si>
+    <t>ENT</t>
   </si>
 </sst>
 </file>
@@ -441,7 +459,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -778,7 +796,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5D25623C-CB7E-43B5-9444-FC757D6B6CE6}">
-  <dimension ref="A1:L109"/>
+  <dimension ref="A1:L112"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.88671875" customWidth="1"/>
@@ -867,7 +885,7 @@
         <v>2</v>
       </c>
       <c r="F4">
-        <f t="shared" ref="F4:F24" si="1">F3+1</f>
+        <f t="shared" ref="F4:F17" si="1">F3+1</f>
         <v>2</v>
       </c>
     </row>
@@ -1114,7 +1132,7 @@
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" t="s">
-        <v>25</v>
+        <v>117</v>
       </c>
       <c r="C17">
         <v>7</v>
@@ -1124,13 +1142,17 @@
       </c>
       <c r="E17">
         <f t="shared" si="0"/>
+        <v>15</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>118</v>
       </c>
       <c r="C18">
         <v>6</v>
@@ -1140,6 +1162,10 @@
       </c>
       <c r="E18">
         <f t="shared" si="0"/>
+        <v>16</v>
+      </c>
+      <c r="F18">
+        <f t="shared" ref="F18:F29" si="2">F17+1</f>
         <v>16</v>
       </c>
     </row>
@@ -1159,8 +1185,8 @@
         <v>17</v>
       </c>
       <c r="F19">
-        <f>F16+1</f>
-        <v>15</v>
+        <f t="shared" si="2"/>
+        <v>17</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
@@ -1179,8 +1205,8 @@
         <v>18</v>
       </c>
       <c r="F20">
-        <f>F19+1</f>
-        <v>16</v>
+        <f t="shared" si="2"/>
+        <v>18</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
@@ -1199,8 +1225,8 @@
         <v>19</v>
       </c>
       <c r="F21">
-        <f>F20+1</f>
-        <v>17</v>
+        <f t="shared" si="2"/>
+        <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -1219,8 +1245,8 @@
         <v>20</v>
       </c>
       <c r="F22">
-        <f>F21+1</f>
-        <v>18</v>
+        <f t="shared" si="2"/>
+        <v>20</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
@@ -1239,8 +1265,8 @@
         <v>21</v>
       </c>
       <c r="F23">
-        <f>F22+1</f>
-        <v>19</v>
+        <f t="shared" si="2"/>
+        <v>21</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
@@ -1259,8 +1285,8 @@
         <v>22</v>
       </c>
       <c r="F24">
-        <f>F23+1</f>
-        <v>20</v>
+        <f t="shared" si="2"/>
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
@@ -1279,8 +1305,8 @@
         <v>23</v>
       </c>
       <c r="F25">
-        <f>F24+1</f>
-        <v>21</v>
+        <f t="shared" si="2"/>
+        <v>23</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
@@ -1299,8 +1325,8 @@
         <v>24</v>
       </c>
       <c r="F26">
-        <f>F25+1</f>
-        <v>22</v>
+        <f t="shared" si="2"/>
+        <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
@@ -1319,8 +1345,8 @@
         <v>25</v>
       </c>
       <c r="F27">
-        <f>F26+1</f>
-        <v>23</v>
+        <f t="shared" si="2"/>
+        <v>25</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
@@ -1339,8 +1365,8 @@
         <v>26</v>
       </c>
       <c r="F28">
-        <f>F27+1</f>
-        <v>24</v>
+        <f t="shared" si="2"/>
+        <v>26</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
@@ -1359,8 +1385,8 @@
         <v>27</v>
       </c>
       <c r="F29">
-        <f>F28+1</f>
-        <v>25</v>
+        <f t="shared" si="2"/>
+        <v>27</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
@@ -1431,7 +1457,7 @@
         <v>4</v>
       </c>
       <c r="E34">
-        <f t="shared" ref="E34:E60" si="2">E33+1</f>
+        <f t="shared" ref="E34:E60" si="3">E33+1</f>
         <v>2</v>
       </c>
     </row>
@@ -1444,7 +1470,7 @@
         <v>8</v>
       </c>
       <c r="E35">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>3</v>
       </c>
     </row>
@@ -1457,7 +1483,7 @@
         <v>10</v>
       </c>
       <c r="E36">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>4</v>
       </c>
     </row>
@@ -1470,7 +1496,7 @@
         <v>20</v>
       </c>
       <c r="E37">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>5</v>
       </c>
     </row>
@@ -1483,7 +1509,7 @@
         <v>40</v>
       </c>
       <c r="E38">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>6</v>
       </c>
     </row>
@@ -1496,7 +1522,7 @@
         <v>80</v>
       </c>
       <c r="E39">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>7</v>
       </c>
     </row>
@@ -1509,7 +1535,7 @@
         <v>1</v>
       </c>
       <c r="E40">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>8</v>
       </c>
     </row>
@@ -1522,7 +1548,7 @@
         <v>2</v>
       </c>
       <c r="E41">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>9</v>
       </c>
     </row>
@@ -1538,11 +1564,11 @@
         <v>4</v>
       </c>
       <c r="E42">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>10</v>
       </c>
       <c r="F42">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="G42" t="s">
         <v>108</v>
@@ -1560,12 +1586,12 @@
         <v>8</v>
       </c>
       <c r="E43">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>11</v>
       </c>
       <c r="F43">
         <f>F42+1</f>
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.3">
@@ -1577,7 +1603,7 @@
         <v>10</v>
       </c>
       <c r="E44">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>12</v>
       </c>
     </row>
@@ -1593,12 +1619,12 @@
         <v>20</v>
       </c>
       <c r="E45">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>13</v>
       </c>
       <c r="F45">
         <f>F43+1</f>
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
@@ -1613,12 +1639,12 @@
         <v>40</v>
       </c>
       <c r="E46">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>14</v>
       </c>
       <c r="F46">
         <f>F45+1</f>
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
@@ -1633,12 +1659,12 @@
         <v>80</v>
       </c>
       <c r="E47">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>15</v>
       </c>
       <c r="F47">
         <f>F46+1</f>
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
@@ -1653,12 +1679,12 @@
         <v>1</v>
       </c>
       <c r="E48">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>16</v>
       </c>
       <c r="F48">
         <f>F47+1</f>
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -1673,12 +1699,12 @@
         <v>2</v>
       </c>
       <c r="E49">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>17</v>
       </c>
       <c r="F49">
         <f>F48+1</f>
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -1693,12 +1719,12 @@
         <v>4</v>
       </c>
       <c r="E50">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>18</v>
       </c>
       <c r="F50">
         <f>F49+1</f>
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
@@ -1710,7 +1736,7 @@
         <v>8</v>
       </c>
       <c r="E51">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>19</v>
       </c>
     </row>
@@ -1723,7 +1749,7 @@
         <v>10</v>
       </c>
       <c r="E52">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>20</v>
       </c>
     </row>
@@ -1736,7 +1762,7 @@
         <v>20</v>
       </c>
       <c r="E53">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>21</v>
       </c>
     </row>
@@ -1749,7 +1775,7 @@
         <v>40</v>
       </c>
       <c r="E54">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>22</v>
       </c>
     </row>
@@ -1765,7 +1791,7 @@
         <v>80</v>
       </c>
       <c r="E55">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>23</v>
       </c>
     </row>
@@ -1781,7 +1807,7 @@
         <v>1</v>
       </c>
       <c r="E56">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>24</v>
       </c>
     </row>
@@ -1797,7 +1823,7 @@
         <v>2</v>
       </c>
       <c r="E57">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>25</v>
       </c>
     </row>
@@ -1813,7 +1839,7 @@
         <v>4</v>
       </c>
       <c r="E58">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>26</v>
       </c>
     </row>
@@ -1829,7 +1855,7 @@
         <v>8</v>
       </c>
       <c r="E59">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>27</v>
       </c>
     </row>
@@ -1845,7 +1871,7 @@
         <v>10</v>
       </c>
       <c r="E60">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>28</v>
       </c>
     </row>
@@ -1882,7 +1908,7 @@
         <v>0</v>
       </c>
       <c r="F62">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
@@ -1902,7 +1928,7 @@
       </c>
       <c r="F63">
         <f>F62+1</f>
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
@@ -1914,7 +1940,7 @@
         <v>4</v>
       </c>
       <c r="E64">
-        <f t="shared" ref="E64:E90" si="3">E63+1</f>
+        <f t="shared" ref="E64:E90" si="4">E63+1</f>
         <v>2</v>
       </c>
     </row>
@@ -1927,7 +1953,7 @@
         <v>8</v>
       </c>
       <c r="E65">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>3</v>
       </c>
     </row>
@@ -1940,7 +1966,7 @@
         <v>10</v>
       </c>
       <c r="E66">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>4</v>
       </c>
     </row>
@@ -1956,12 +1982,12 @@
         <v>20</v>
       </c>
       <c r="E67">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>5</v>
       </c>
       <c r="F67">
         <f>F63+1</f>
-        <v>36</v>
+        <v>38</v>
       </c>
     </row>
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
@@ -1976,12 +2002,12 @@
         <v>40</v>
       </c>
       <c r="E68">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>6</v>
       </c>
       <c r="F68">
         <f>F67+1</f>
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
@@ -1996,15 +2022,15 @@
         <v>80</v>
       </c>
       <c r="E69">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>7</v>
       </c>
       <c r="F69">
         <f>F68+1</f>
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="G69">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="H69" t="s">
         <v>110</v>
@@ -2019,7 +2045,7 @@
         <v>1</v>
       </c>
       <c r="E70">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>8</v>
       </c>
     </row>
@@ -2032,7 +2058,7 @@
         <v>2</v>
       </c>
       <c r="E71">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>9</v>
       </c>
     </row>
@@ -2048,11 +2074,11 @@
         <v>4</v>
       </c>
       <c r="E72">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>10</v>
       </c>
       <c r="F72">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
@@ -2067,15 +2093,15 @@
         <v>8</v>
       </c>
       <c r="E73">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>11</v>
       </c>
       <c r="F73">
         <f>F72+1</f>
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="G73">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H73" t="s">
         <v>111</v>
@@ -2093,11 +2119,11 @@
         <v>10</v>
       </c>
       <c r="E74">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>12</v>
       </c>
       <c r="F74">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
@@ -2112,12 +2138,12 @@
         <v>20</v>
       </c>
       <c r="E75">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>13</v>
       </c>
       <c r="F75">
         <f>F74+1</f>
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="76" spans="1:8" x14ac:dyDescent="0.3">
@@ -2129,7 +2155,7 @@
         <v>40</v>
       </c>
       <c r="E76">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>14</v>
       </c>
     </row>
@@ -2145,12 +2171,12 @@
         <v>80</v>
       </c>
       <c r="E77">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>15</v>
       </c>
       <c r="F77">
         <f>F75+1</f>
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
@@ -2165,12 +2191,12 @@
         <v>1</v>
       </c>
       <c r="E78">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>16</v>
       </c>
       <c r="F78">
-        <f>F77+1</f>
-        <v>46</v>
+        <f t="shared" ref="F78:F86" si="5">F77+1</f>
+        <v>48</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
@@ -2185,12 +2211,12 @@
         <v>2</v>
       </c>
       <c r="E79">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>17</v>
       </c>
       <c r="F79">
-        <f>F78+1</f>
-        <v>47</v>
+        <f t="shared" si="5"/>
+        <v>49</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
@@ -2205,12 +2231,12 @@
         <v>4</v>
       </c>
       <c r="E80">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>18</v>
       </c>
       <c r="F80">
-        <f>F79+1</f>
-        <v>48</v>
+        <f t="shared" si="5"/>
+        <v>50</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
@@ -2225,12 +2251,12 @@
         <v>8</v>
       </c>
       <c r="E81">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>19</v>
       </c>
       <c r="F81">
-        <f>F80+1</f>
-        <v>49</v>
+        <f t="shared" si="5"/>
+        <v>51</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
@@ -2245,12 +2271,12 @@
         <v>10</v>
       </c>
       <c r="E82">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>20</v>
       </c>
       <c r="F82">
-        <f>F81+1</f>
-        <v>50</v>
+        <f t="shared" si="5"/>
+        <v>52</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
@@ -2265,12 +2291,12 @@
         <v>20</v>
       </c>
       <c r="E83">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>21</v>
       </c>
       <c r="F83">
-        <f>F82+1</f>
-        <v>51</v>
+        <f t="shared" si="5"/>
+        <v>53</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
@@ -2285,12 +2311,12 @@
         <v>40</v>
       </c>
       <c r="E84">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>22</v>
       </c>
       <c r="F84">
-        <f>F83+1</f>
-        <v>52</v>
+        <f t="shared" si="5"/>
+        <v>54</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
@@ -2305,12 +2331,12 @@
         <v>80</v>
       </c>
       <c r="E85">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>23</v>
       </c>
       <c r="F85">
-        <f>F84+1</f>
-        <v>53</v>
+        <f t="shared" si="5"/>
+        <v>55</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
@@ -2325,12 +2351,12 @@
         <v>1</v>
       </c>
       <c r="E86">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>24</v>
       </c>
       <c r="F86">
-        <f>F85+1</f>
-        <v>54</v>
+        <f t="shared" si="5"/>
+        <v>56</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.3">
@@ -2345,7 +2371,7 @@
         <v>2</v>
       </c>
       <c r="E87">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>25</v>
       </c>
     </row>
@@ -2361,7 +2387,7 @@
         <v>4</v>
       </c>
       <c r="E88">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>26</v>
       </c>
     </row>
@@ -2377,7 +2403,7 @@
         <v>8</v>
       </c>
       <c r="E89">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>27</v>
       </c>
     </row>
@@ -2393,7 +2419,7 @@
         <v>10</v>
       </c>
       <c r="E90">
-        <f t="shared" si="3"/>
+        <f t="shared" si="4"/>
         <v>28</v>
       </c>
     </row>
@@ -2413,122 +2439,161 @@
         <v>29</v>
       </c>
     </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A92" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B92" t="s">
+        <v>113</v>
+      </c>
+      <c r="F92">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A93" s="4"/>
+      <c r="B93" t="s">
+        <v>114</v>
+      </c>
+      <c r="F93">
+        <v>58</v>
+      </c>
+    </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A94" t="s">
+      <c r="A94" s="4"/>
+      <c r="B94" t="s">
+        <v>115</v>
+      </c>
+      <c r="F94">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A95" s="4"/>
+      <c r="B95" t="s">
+        <v>116</v>
+      </c>
+      <c r="F95">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="97" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
         <v>68</v>
       </c>
-      <c r="B94" t="s">
+      <c r="B97" t="s">
         <v>69</v>
       </c>
-      <c r="C94" s="2" t="s">
+      <c r="C97" s="2" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="B95" t="s">
+    <row r="98" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B98" t="s">
         <v>79</v>
       </c>
-      <c r="C95" s="2" t="s">
+      <c r="C98" s="2" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A96" t="s">
+    <row r="99" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A99" t="s">
         <v>70</v>
       </c>
-      <c r="B96" t="s">
+      <c r="B99" t="s">
         <v>78</v>
       </c>
-      <c r="C96" s="2" t="s">
+      <c r="C99" s="2" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B97" t="s">
+    <row r="100" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B100" t="s">
         <v>80</v>
       </c>
-      <c r="C97" s="2" t="s">
+      <c r="C100" s="2" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A98" t="s">
+    <row r="101" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
         <v>71</v>
       </c>
-      <c r="B98" t="s">
+      <c r="B101" t="s">
         <v>81</v>
       </c>
-      <c r="C98" s="2" t="s">
+      <c r="C101" s="2" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="B99" t="s">
+    <row r="102" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="B102" t="s">
         <v>82</v>
       </c>
-      <c r="C99" s="2" t="s">
+      <c r="C102" s="2" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A102" s="1" t="s">
+    <row r="105" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A105" s="1" t="s">
         <v>83</v>
-      </c>
-    </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A103" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B103" s="3"/>
-      <c r="C103" s="3"/>
-      <c r="D103" s="3"/>
-      <c r="E103" s="3"/>
-      <c r="F103" s="3" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A104" s="3" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A105" s="3" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A106" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
+      </c>
+      <c r="B106" s="3"/>
+      <c r="C106" s="3"/>
+      <c r="D106" s="3"/>
+      <c r="E106" s="3"/>
+      <c r="F106" s="3" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A107" s="3" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="108" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A108" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="109" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A109" s="3" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="110" spans="1:12" x14ac:dyDescent="0.3">
+      <c r="A110" s="3" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="109" spans="1:12" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A109" s="5" t="s">
+    <row r="112" spans="1:12" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A112" s="5" t="s">
         <v>112</v>
       </c>
-      <c r="B109" s="5"/>
-      <c r="C109" s="5"/>
-      <c r="D109" s="5"/>
-      <c r="E109" s="5"/>
-      <c r="F109" s="5"/>
-      <c r="G109" s="5"/>
-      <c r="H109" s="5"/>
-      <c r="I109" s="5"/>
-      <c r="J109" s="5"/>
-      <c r="K109" s="5"/>
-      <c r="L109" s="5"/>
+      <c r="B112" s="5"/>
+      <c r="C112" s="5"/>
+      <c r="D112" s="5"/>
+      <c r="E112" s="5"/>
+      <c r="F112" s="5"/>
+      <c r="G112" s="5"/>
+      <c r="H112" s="5"/>
+      <c r="I112" s="5"/>
+      <c r="J112" s="5"/>
+      <c r="K112" s="5"/>
+      <c r="L112" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
+  <mergeCells count="5">
     <mergeCell ref="A2:A31"/>
     <mergeCell ref="A32:A61"/>
     <mergeCell ref="A62:A91"/>
-    <mergeCell ref="A109:L109"/>
+    <mergeCell ref="A112:L112"/>
+    <mergeCell ref="A92:A95"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Minor debugging and adding of buttons. Adding the ddi sketch, also built on the cockpit library.
</commit_message>
<xml_diff>
--- a/Button tables.xlsx
+++ b/Button tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\git\cockpit_arduino\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B58493AB-5991-4EBB-BF6C-078A1D3566E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E558506-15F2-4FBC-BA01-BBD2D955D7B3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60450" yWindow="12945" windowWidth="30420" windowHeight="18330" xr2:uid="{B42DDCD9-64C5-4A29-BEC7-73E9BF8FAFC9}"/>
+    <workbookView xWindow="1020" yWindow="4140" windowWidth="15636" windowHeight="18336" xr2:uid="{B42DDCD9-64C5-4A29-BEC7-73E9BF8FAFC9}"/>
   </bookViews>
   <sheets>
     <sheet name="Radio Arduino" sheetId="2" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="119">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="122">
   <si>
     <t>Key</t>
   </si>
@@ -117,12 +117,6 @@
     <t>-</t>
   </si>
   <si>
-    <t>DDI Left = ?</t>
-  </si>
-  <si>
-    <t>DDI Right = ?</t>
-  </si>
-  <si>
     <t>Radio = 0</t>
   </si>
   <si>
@@ -333,12 +327,6 @@
     <t>ADF Up</t>
   </si>
   <si>
-    <t>HDG Switch On</t>
-  </si>
-  <si>
-    <t>CRS Switch On</t>
-  </si>
-  <si>
     <t>Func sel 1 A/P</t>
   </si>
   <si>
@@ -394,6 +382,27 @@
   </si>
   <si>
     <t>ENT</t>
+  </si>
+  <si>
+    <t>DDI Left = 2</t>
+  </si>
+  <si>
+    <t>DDI Bottom = 1</t>
+  </si>
+  <si>
+    <t>DDI Right = 0</t>
+  </si>
+  <si>
+    <t>CRS Switch Left</t>
+  </si>
+  <si>
+    <t>HDG Switch Right</t>
+  </si>
+  <si>
+    <t>HDG Switch Left</t>
+  </si>
+  <si>
+    <t>CRS Switch Right</t>
   </si>
 </sst>
 </file>
@@ -814,10 +823,10 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>1</v>
@@ -826,15 +835,15 @@
         <v>2</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="C2">
         <v>8</v>
@@ -852,7 +861,7 @@
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
       <c r="B3" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="C3">
         <v>8</v>
@@ -872,7 +881,7 @@
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
       <c r="B4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C4">
         <v>8</v>
@@ -892,7 +901,7 @@
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="C5">
         <v>8</v>
@@ -912,7 +921,7 @@
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C6">
         <v>8</v>
@@ -932,7 +941,7 @@
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="C7">
         <v>8</v>
@@ -952,7 +961,7 @@
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C8">
         <v>8</v>
@@ -972,7 +981,7 @@
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C9">
         <v>8</v>
@@ -992,7 +1001,7 @@
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C10">
         <v>7</v>
@@ -1012,7 +1021,7 @@
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C11">
         <v>7</v>
@@ -1032,7 +1041,7 @@
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C12">
         <v>7</v>
@@ -1052,7 +1061,7 @@
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C13">
         <v>7</v>
@@ -1072,7 +1081,7 @@
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="C14">
         <v>7</v>
@@ -1092,7 +1101,7 @@
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="C15">
         <v>7</v>
@@ -1112,7 +1121,7 @@
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C16">
         <v>7</v>
@@ -1132,7 +1141,7 @@
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" t="s">
-        <v>117</v>
+        <v>113</v>
       </c>
       <c r="C17">
         <v>7</v>
@@ -1152,7 +1161,7 @@
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="C18">
         <v>6</v>
@@ -1172,7 +1181,7 @@
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C19">
         <v>6</v>
@@ -1192,7 +1201,7 @@
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
       <c r="B20" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C20">
         <v>6</v>
@@ -1212,7 +1221,7 @@
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="C21">
         <v>6</v>
@@ -1232,7 +1241,7 @@
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
       <c r="B22" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
       <c r="C22">
         <v>6</v>
@@ -1252,7 +1261,7 @@
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
       <c r="B23" t="s">
-        <v>104</v>
+        <v>100</v>
       </c>
       <c r="C23">
         <v>6</v>
@@ -1272,7 +1281,7 @@
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="4"/>
       <c r="B24" t="s">
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="C24">
         <v>6</v>
@@ -1292,7 +1301,7 @@
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="4"/>
       <c r="B25" t="s">
-        <v>102</v>
+        <v>98</v>
       </c>
       <c r="C25">
         <v>6</v>
@@ -1312,7 +1321,7 @@
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" t="s">
-        <v>101</v>
+        <v>97</v>
       </c>
       <c r="C26">
         <v>5</v>
@@ -1332,7 +1341,7 @@
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="4"/>
       <c r="B27" t="s">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="C27">
         <v>5</v>
@@ -1352,7 +1361,7 @@
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
       <c r="B28" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="C28">
         <v>5</v>
@@ -1372,7 +1381,7 @@
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="C29">
         <v>5</v>
@@ -1423,7 +1432,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C32">
         <v>19</v>
@@ -1555,7 +1564,7 @@
     <row r="42" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A42" s="4"/>
       <c r="B42" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C42">
         <v>18</v>
@@ -1571,13 +1580,13 @@
         <v>28</v>
       </c>
       <c r="G42" t="s">
-        <v>108</v>
+        <v>104</v>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A43" s="4"/>
       <c r="B43" t="s">
-        <v>109</v>
+        <v>105</v>
       </c>
       <c r="C43">
         <v>18</v>
@@ -1610,7 +1619,7 @@
     <row r="45" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A45" s="4"/>
       <c r="B45" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C45">
         <v>18</v>
@@ -1630,7 +1639,7 @@
     <row r="46" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A46" s="4"/>
       <c r="B46" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C46">
         <v>18</v>
@@ -1649,9 +1658,6 @@
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A47" s="4"/>
-      <c r="B47" t="s">
-        <v>91</v>
-      </c>
       <c r="C47">
         <v>18</v>
       </c>
@@ -1661,16 +1667,12 @@
       <c r="E47">
         <f t="shared" si="3"/>
         <v>15</v>
-      </c>
-      <c r="F47">
-        <f>F46+1</f>
-        <v>32</v>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A48" s="4"/>
       <c r="B48" t="s">
-        <v>50</v>
+        <v>89</v>
       </c>
       <c r="C48">
         <v>17</v>
@@ -1683,14 +1685,14 @@
         <v>16</v>
       </c>
       <c r="F48">
-        <f>F47+1</f>
-        <v>33</v>
+        <f>F46+1</f>
+        <v>32</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="4"/>
       <c r="B49" t="s">
-        <v>92</v>
+        <v>48</v>
       </c>
       <c r="C49">
         <v>17</v>
@@ -1704,13 +1706,13 @@
       </c>
       <c r="F49">
         <f>F48+1</f>
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="4"/>
       <c r="B50" t="s">
-        <v>51</v>
+        <v>90</v>
       </c>
       <c r="C50">
         <v>17</v>
@@ -1724,11 +1726,14 @@
       </c>
       <c r="F50">
         <f>F49+1</f>
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="4"/>
+      <c r="B51" t="s">
+        <v>49</v>
+      </c>
       <c r="C51">
         <v>17</v>
       </c>
@@ -1738,6 +1743,10 @@
       <c r="E51">
         <f t="shared" si="3"/>
         <v>19</v>
+      </c>
+      <c r="F51">
+        <f>F50+1</f>
+        <v>35</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
@@ -1893,10 +1902,10 @@
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B62" t="s">
-        <v>99</v>
+        <v>120</v>
       </c>
       <c r="C62">
         <v>30</v>
@@ -1914,7 +1923,7 @@
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="4"/>
       <c r="B63" t="s">
-        <v>98</v>
+        <v>119</v>
       </c>
       <c r="C63">
         <v>30</v>
@@ -1933,6 +1942,9 @@
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="4"/>
+      <c r="B64" t="s">
+        <v>121</v>
+      </c>
       <c r="C64">
         <v>30</v>
       </c>
@@ -1943,9 +1955,15 @@
         <f t="shared" ref="E64:E90" si="4">E63+1</f>
         <v>2</v>
       </c>
+      <c r="F64">
+        <v>57</v>
+      </c>
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="4"/>
+      <c r="B65" t="s">
+        <v>118</v>
+      </c>
       <c r="C65">
         <v>30</v>
       </c>
@@ -1955,6 +1973,9 @@
       <c r="E65">
         <f t="shared" si="4"/>
         <v>3</v>
+      </c>
+      <c r="F65">
+        <v>58</v>
       </c>
     </row>
     <row r="66" spans="1:8" x14ac:dyDescent="0.3">
@@ -1973,7 +1994,7 @@
     <row r="67" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A67" s="4"/>
       <c r="B67" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="C67">
         <v>30</v>
@@ -1993,7 +2014,7 @@
     <row r="68" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A68" s="4"/>
       <c r="B68" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="C68">
         <v>30</v>
@@ -2013,7 +2034,7 @@
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="4"/>
       <c r="B69" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="C69">
         <v>30</v>
@@ -2033,7 +2054,7 @@
         <v>41</v>
       </c>
       <c r="H69" t="s">
-        <v>110</v>
+        <v>106</v>
       </c>
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
@@ -2065,7 +2086,7 @@
     <row r="72" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A72" s="4"/>
       <c r="B72" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C72">
         <v>29</v>
@@ -2084,7 +2105,7 @@
     <row r="73" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A73" s="4"/>
       <c r="B73" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C73">
         <v>29</v>
@@ -2104,13 +2125,13 @@
         <v>44</v>
       </c>
       <c r="H73" t="s">
-        <v>111</v>
+        <v>107</v>
       </c>
     </row>
     <row r="74" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A74" s="4"/>
       <c r="B74" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="C74">
         <v>29</v>
@@ -2129,7 +2150,7 @@
     <row r="75" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A75" s="4"/>
       <c r="B75" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="C75">
         <v>29</v>
@@ -2162,7 +2183,7 @@
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="4"/>
       <c r="B77" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C77">
         <v>29</v>
@@ -2182,7 +2203,7 @@
     <row r="78" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A78" s="4"/>
       <c r="B78" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="C78">
         <v>28</v>
@@ -2202,7 +2223,7 @@
     <row r="79" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A79" s="4"/>
       <c r="B79" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="C79">
         <v>28</v>
@@ -2222,7 +2243,7 @@
     <row r="80" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A80" s="4"/>
       <c r="B80" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="C80">
         <v>28</v>
@@ -2242,7 +2263,7 @@
     <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="4"/>
       <c r="B81" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="C81">
         <v>28</v>
@@ -2262,7 +2283,7 @@
     <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="4"/>
       <c r="B82" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C82">
         <v>28</v>
@@ -2282,7 +2303,7 @@
     <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="4"/>
       <c r="B83" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C83">
         <v>28</v>
@@ -2302,7 +2323,7 @@
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="4"/>
       <c r="B84" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C84">
         <v>28</v>
@@ -2322,7 +2343,7 @@
     <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="4"/>
       <c r="B85" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C85">
         <v>28</v>
@@ -2342,7 +2363,7 @@
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="4"/>
       <c r="B86" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="C86">
         <v>27</v>
@@ -2441,139 +2462,139 @@
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B92" t="s">
-        <v>113</v>
+        <v>109</v>
       </c>
       <c r="F92">
-        <v>57</v>
+        <v>90</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="4"/>
       <c r="B93" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="F93">
-        <v>58</v>
+        <v>91</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="4"/>
       <c r="B94" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="F94">
-        <v>59</v>
+        <v>92</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="4"/>
       <c r="B95" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
       <c r="F95">
-        <v>60</v>
+        <v>93</v>
       </c>
     </row>
     <row r="97" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B97" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="98" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B98" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C98" s="2" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="99" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B99" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="100" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B100" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="C100" s="2" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
     </row>
     <row r="101" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B101" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="C101" s="2" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="102" spans="1:12" x14ac:dyDescent="0.3">
       <c r="B102" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C102" s="2" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="105" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="106" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A106" s="3" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B106" s="3"/>
       <c r="C106" s="3"/>
       <c r="D106" s="3"/>
       <c r="E106" s="3"/>
       <c r="F106" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="107" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A107" s="3" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="108" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A108" s="3" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="109" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A109" s="3" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="110" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A110" s="3" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
     </row>
     <row r="112" spans="1:12" ht="49.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A112" s="5" t="s">
-        <v>112</v>
+        <v>108</v>
       </c>
       <c r="B112" s="5"/>
       <c r="C112" s="5"/>
@@ -2602,16 +2623,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09AF7111-1B37-497D-B08D-3EB3AFC0EDCF}">
-  <dimension ref="A1:D91"/>
+  <dimension ref="A1:F106"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="15.88671875" customWidth="1"/>
     <col min="2" max="2" width="29" customWidth="1"/>
-    <col min="3" max="3" width="15" customWidth="1"/>
-    <col min="4" max="4" width="24.33203125" customWidth="1"/>
+    <col min="3" max="4" width="8" customWidth="1"/>
+    <col min="5" max="5" width="15" customWidth="1"/>
+    <col min="6" max="6" width="24.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -2619,1187 +2641,1767 @@
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>26</v>
+        <v>117</v>
       </c>
       <c r="B2" t="s">
         <v>4</v>
       </c>
       <c r="C2">
+        <v>8</v>
+      </c>
+      <c r="D2">
+        <v>1</v>
+      </c>
+      <c r="E2">
         <v>0</v>
       </c>
-      <c r="D2">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F2">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3">
-        <f>C2+1</f>
+        <v>8</v>
+      </c>
+      <c r="D3">
+        <v>2</v>
+      </c>
+      <c r="E3">
+        <f>E2+1</f>
         <v>1</v>
       </c>
-      <c r="D3">
-        <f>D2+1</f>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F3">
+        <f>F2+1</f>
+        <v>24</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="4"/>
       <c r="B4" t="s">
         <v>6</v>
       </c>
       <c r="C4">
-        <f t="shared" ref="C4:C30" si="0">C3+1</f>
+        <v>8</v>
+      </c>
+      <c r="D4">
+        <v>4</v>
+      </c>
+      <c r="E4">
+        <f t="shared" ref="E4:E30" si="0">E3+1</f>
         <v>2</v>
       </c>
-      <c r="D4">
-        <f t="shared" ref="D4:D24" si="1">D3+1</f>
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F4">
+        <f t="shared" ref="F4:F24" si="1">F3+1</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="4"/>
       <c r="B5" t="s">
         <v>7</v>
       </c>
       <c r="C5">
+        <v>8</v>
+      </c>
+      <c r="D5">
+        <v>8</v>
+      </c>
+      <c r="E5">
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="D5">
+      <c r="F5">
         <f t="shared" si="1"/>
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" t="s">
         <v>8</v>
       </c>
       <c r="C6">
+        <v>8</v>
+      </c>
+      <c r="D6">
+        <v>10</v>
+      </c>
+      <c r="E6">
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="D6">
+      <c r="F6">
         <f t="shared" si="1"/>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" t="s">
         <v>9</v>
       </c>
       <c r="C7">
+        <v>8</v>
+      </c>
+      <c r="D7">
+        <v>20</v>
+      </c>
+      <c r="E7">
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="D7">
+      <c r="F7">
         <f t="shared" si="1"/>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" t="s">
         <v>10</v>
       </c>
       <c r="C8">
+        <v>8</v>
+      </c>
+      <c r="D8">
+        <v>40</v>
+      </c>
+      <c r="E8">
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="D8">
+      <c r="F8">
         <f t="shared" si="1"/>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" t="s">
         <v>11</v>
       </c>
       <c r="C9">
+        <v>8</v>
+      </c>
+      <c r="D9">
+        <v>80</v>
+      </c>
+      <c r="E9">
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="D9">
+      <c r="F9">
         <f t="shared" si="1"/>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" t="s">
         <v>12</v>
       </c>
       <c r="C10">
-        <f t="shared" si="0"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <f t="shared" si="0"/>
+        <v>8</v>
+      </c>
+      <c r="F10">
         <f t="shared" si="1"/>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" t="s">
         <v>13</v>
       </c>
       <c r="C11">
+        <v>7</v>
+      </c>
+      <c r="D11">
+        <v>2</v>
+      </c>
+      <c r="E11">
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="D11">
+      <c r="F11">
         <f t="shared" si="1"/>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" t="s">
         <v>14</v>
       </c>
       <c r="C12">
+        <v>7</v>
+      </c>
+      <c r="D12">
+        <v>4</v>
+      </c>
+      <c r="E12">
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="D12">
+      <c r="F12">
         <f t="shared" si="1"/>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" t="s">
         <v>15</v>
       </c>
       <c r="C13">
+        <v>7</v>
+      </c>
+      <c r="D13">
+        <v>8</v>
+      </c>
+      <c r="E13">
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="D13">
+      <c r="F13">
         <f t="shared" si="1"/>
-        <v>11</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" t="s">
         <v>16</v>
       </c>
       <c r="C14">
+        <v>7</v>
+      </c>
+      <c r="D14">
+        <v>10</v>
+      </c>
+      <c r="E14">
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="D14">
+      <c r="F14">
         <f t="shared" si="1"/>
-        <v>12</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" t="s">
         <v>17</v>
       </c>
       <c r="C15">
+        <v>7</v>
+      </c>
+      <c r="D15">
+        <v>20</v>
+      </c>
+      <c r="E15">
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="D15">
+      <c r="F15">
         <f t="shared" si="1"/>
-        <v>13</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" t="s">
         <v>18</v>
       </c>
       <c r="C16">
+        <v>7</v>
+      </c>
+      <c r="D16">
+        <v>40</v>
+      </c>
+      <c r="E16">
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="D16">
+      <c r="F16">
         <f t="shared" si="1"/>
-        <v>14</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" t="s">
         <v>19</v>
       </c>
       <c r="C17">
+        <v>7</v>
+      </c>
+      <c r="D17">
+        <v>80</v>
+      </c>
+      <c r="E17">
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="D17">
+      <c r="F17">
         <f t="shared" si="1"/>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" t="s">
         <v>20</v>
       </c>
       <c r="C18">
+        <v>6</v>
+      </c>
+      <c r="D18">
+        <v>1</v>
+      </c>
+      <c r="E18">
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="D18">
+      <c r="F18">
         <f t="shared" si="1"/>
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" t="s">
         <v>21</v>
       </c>
       <c r="C19">
+        <v>6</v>
+      </c>
+      <c r="D19">
+        <v>2</v>
+      </c>
+      <c r="E19">
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="D19">
+      <c r="F19">
         <f t="shared" si="1"/>
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
       <c r="B20" t="s">
         <v>22</v>
       </c>
       <c r="C20">
+        <v>6</v>
+      </c>
+      <c r="D20">
+        <v>4</v>
+      </c>
+      <c r="E20">
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="D20">
+      <c r="F20">
         <f t="shared" si="1"/>
-        <v>18</v>
-      </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" t="s">
         <v>23</v>
       </c>
       <c r="C21">
+        <v>6</v>
+      </c>
+      <c r="D21">
+        <v>8</v>
+      </c>
+      <c r="E21">
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="D21">
+      <c r="F21">
         <f t="shared" si="1"/>
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
       <c r="B22" t="s">
         <v>24</v>
       </c>
       <c r="C22">
+        <v>6</v>
+      </c>
+      <c r="D22">
+        <v>10</v>
+      </c>
+      <c r="E22">
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="D22">
+      <c r="F22">
         <f t="shared" si="1"/>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
       <c r="B23" t="s">
         <v>24</v>
       </c>
       <c r="C23">
+        <v>6</v>
+      </c>
+      <c r="D23">
+        <v>20</v>
+      </c>
+      <c r="E23">
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="D23">
+      <c r="F23">
         <f t="shared" si="1"/>
-        <v>21</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="4"/>
       <c r="B24" t="s">
         <v>24</v>
       </c>
       <c r="C24">
+        <v>6</v>
+      </c>
+      <c r="D24">
+        <v>40</v>
+      </c>
+      <c r="E24">
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="D24">
+      <c r="F24">
         <f t="shared" si="1"/>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="4"/>
       <c r="B25" t="s">
         <v>25</v>
       </c>
       <c r="C25">
+        <v>6</v>
+      </c>
+      <c r="D25">
+        <v>80</v>
+      </c>
+      <c r="E25">
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" t="s">
         <v>25</v>
       </c>
       <c r="C26">
+        <v>5</v>
+      </c>
+      <c r="D26">
+        <v>1</v>
+      </c>
+      <c r="E26">
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="4"/>
       <c r="B27" t="s">
         <v>25</v>
       </c>
       <c r="C27">
+        <v>5</v>
+      </c>
+      <c r="D27">
+        <v>2</v>
+      </c>
+      <c r="E27">
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
       <c r="B28" t="s">
         <v>25</v>
       </c>
       <c r="C28">
+        <v>5</v>
+      </c>
+      <c r="D28">
+        <v>4</v>
+      </c>
+      <c r="E28">
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" t="s">
         <v>25</v>
       </c>
       <c r="C29">
+        <v>5</v>
+      </c>
+      <c r="D29">
+        <v>8</v>
+      </c>
+      <c r="E29">
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="4"/>
       <c r="B30" t="s">
         <v>25</v>
       </c>
       <c r="C30">
+        <v>5</v>
+      </c>
+      <c r="D30">
+        <v>10</v>
+      </c>
+      <c r="E30">
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="4"/>
       <c r="B31" t="s">
         <v>25</v>
       </c>
       <c r="C31">
-        <f>C30+1</f>
+        <v>5</v>
+      </c>
+      <c r="D31">
+        <v>20</v>
+      </c>
+      <c r="E31">
+        <f>E30+1</f>
         <v>29</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>27</v>
+        <v>116</v>
       </c>
       <c r="B32" t="s">
         <v>4</v>
       </c>
       <c r="C32">
+        <v>19</v>
+      </c>
+      <c r="D32">
+        <v>1</v>
+      </c>
+      <c r="E32">
         <v>0</v>
       </c>
-      <c r="D32">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F32">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="4"/>
       <c r="B33" t="s">
         <v>5</v>
       </c>
       <c r="C33">
-        <f>C32+1</f>
+        <v>19</v>
+      </c>
+      <c r="D33">
+        <v>2</v>
+      </c>
+      <c r="E33">
+        <f>E32+1</f>
         <v>1</v>
       </c>
-      <c r="D33">
-        <f>D32+1</f>
-        <v>24</v>
-      </c>
-    </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F33">
+        <f>F32+1</f>
+        <v>47</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="4"/>
       <c r="B34" t="s">
         <v>6</v>
       </c>
       <c r="C34">
-        <f t="shared" ref="C34:C60" si="2">C33+1</f>
+        <v>19</v>
+      </c>
+      <c r="D34">
+        <v>4</v>
+      </c>
+      <c r="E34">
+        <f t="shared" ref="E34:E60" si="2">E33+1</f>
         <v>2</v>
       </c>
-      <c r="D34">
-        <f t="shared" ref="D34:D54" si="3">D33+1</f>
-        <v>25</v>
-      </c>
-    </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F34">
+        <f t="shared" ref="F34:F54" si="3">F33+1</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="4"/>
       <c r="B35" t="s">
         <v>7</v>
       </c>
       <c r="C35">
+        <v>19</v>
+      </c>
+      <c r="D35">
+        <v>8</v>
+      </c>
+      <c r="E35">
         <f t="shared" si="2"/>
         <v>3</v>
       </c>
-      <c r="D35">
-        <f t="shared" si="3"/>
-        <v>26</v>
-      </c>
-    </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F35">
+        <f t="shared" si="3"/>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="4"/>
       <c r="B36" t="s">
         <v>8</v>
       </c>
       <c r="C36">
+        <v>19</v>
+      </c>
+      <c r="D36">
+        <v>10</v>
+      </c>
+      <c r="E36">
         <f t="shared" si="2"/>
         <v>4</v>
       </c>
-      <c r="D36">
-        <f t="shared" si="3"/>
-        <v>27</v>
-      </c>
-    </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F36">
+        <f t="shared" si="3"/>
+        <v>50</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="4"/>
       <c r="B37" t="s">
         <v>9</v>
       </c>
       <c r="C37">
+        <v>19</v>
+      </c>
+      <c r="D37">
+        <v>20</v>
+      </c>
+      <c r="E37">
         <f t="shared" si="2"/>
         <v>5</v>
       </c>
-      <c r="D37">
-        <f t="shared" si="3"/>
-        <v>28</v>
-      </c>
-    </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F37">
+        <f t="shared" si="3"/>
+        <v>51</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="4"/>
       <c r="B38" t="s">
         <v>10</v>
       </c>
       <c r="C38">
+        <v>19</v>
+      </c>
+      <c r="D38">
+        <v>40</v>
+      </c>
+      <c r="E38">
         <f t="shared" si="2"/>
         <v>6</v>
       </c>
-      <c r="D38">
-        <f t="shared" si="3"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F38">
+        <f t="shared" si="3"/>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" t="s">
         <v>11</v>
       </c>
       <c r="C39">
+        <v>19</v>
+      </c>
+      <c r="D39">
+        <v>80</v>
+      </c>
+      <c r="E39">
         <f t="shared" si="2"/>
         <v>7</v>
       </c>
-      <c r="D39">
-        <f t="shared" si="3"/>
-        <v>30</v>
-      </c>
-    </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F39">
+        <f t="shared" si="3"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" t="s">
         <v>12</v>
       </c>
       <c r="C40">
+        <v>18</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+      <c r="E40">
         <f t="shared" si="2"/>
         <v>8</v>
       </c>
-      <c r="D40">
-        <f t="shared" si="3"/>
-        <v>31</v>
-      </c>
-    </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F40">
+        <f t="shared" si="3"/>
+        <v>54</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" t="s">
         <v>13</v>
       </c>
       <c r="C41">
+        <v>18</v>
+      </c>
+      <c r="D41">
+        <v>2</v>
+      </c>
+      <c r="E41">
         <f t="shared" si="2"/>
         <v>9</v>
       </c>
-      <c r="D41">
-        <f t="shared" si="3"/>
-        <v>32</v>
-      </c>
-    </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F41">
+        <f t="shared" si="3"/>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="4"/>
       <c r="B42" t="s">
         <v>14</v>
       </c>
       <c r="C42">
+        <v>18</v>
+      </c>
+      <c r="D42">
+        <v>4</v>
+      </c>
+      <c r="E42">
         <f t="shared" si="2"/>
         <v>10</v>
       </c>
-      <c r="D42">
-        <f t="shared" si="3"/>
-        <v>33</v>
-      </c>
-    </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F42">
+        <f t="shared" si="3"/>
+        <v>56</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="4"/>
       <c r="B43" t="s">
         <v>15</v>
       </c>
       <c r="C43">
+        <v>18</v>
+      </c>
+      <c r="D43">
+        <v>8</v>
+      </c>
+      <c r="E43">
         <f t="shared" si="2"/>
         <v>11</v>
       </c>
-      <c r="D43">
-        <f t="shared" si="3"/>
-        <v>34</v>
-      </c>
-    </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F43">
+        <f t="shared" si="3"/>
+        <v>57</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="4"/>
       <c r="B44" t="s">
         <v>16</v>
       </c>
       <c r="C44">
+        <v>18</v>
+      </c>
+      <c r="D44">
+        <v>10</v>
+      </c>
+      <c r="E44">
         <f t="shared" si="2"/>
         <v>12</v>
       </c>
-      <c r="D44">
-        <f t="shared" si="3"/>
-        <v>35</v>
-      </c>
-    </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F44">
+        <f t="shared" si="3"/>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="4"/>
       <c r="B45" t="s">
         <v>17</v>
       </c>
       <c r="C45">
+        <v>18</v>
+      </c>
+      <c r="D45">
+        <v>20</v>
+      </c>
+      <c r="E45">
         <f t="shared" si="2"/>
         <v>13</v>
       </c>
-      <c r="D45">
-        <f t="shared" si="3"/>
-        <v>36</v>
-      </c>
-    </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F45">
+        <f t="shared" si="3"/>
+        <v>59</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="4"/>
       <c r="B46" t="s">
         <v>18</v>
       </c>
       <c r="C46">
+        <v>18</v>
+      </c>
+      <c r="D46">
+        <v>40</v>
+      </c>
+      <c r="E46">
         <f t="shared" si="2"/>
         <v>14</v>
       </c>
-      <c r="D46">
-        <f t="shared" si="3"/>
-        <v>37</v>
-      </c>
-    </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F46">
+        <f t="shared" si="3"/>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="4"/>
       <c r="B47" t="s">
         <v>19</v>
       </c>
       <c r="C47">
+        <v>18</v>
+      </c>
+      <c r="D47">
+        <v>80</v>
+      </c>
+      <c r="E47">
         <f t="shared" si="2"/>
         <v>15</v>
       </c>
-      <c r="D47">
-        <f t="shared" si="3"/>
-        <v>38</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F47">
+        <f t="shared" si="3"/>
+        <v>61</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="4"/>
       <c r="B48" t="s">
         <v>20</v>
       </c>
       <c r="C48">
+        <v>17</v>
+      </c>
+      <c r="D48">
+        <v>1</v>
+      </c>
+      <c r="E48">
         <f t="shared" si="2"/>
         <v>16</v>
       </c>
-      <c r="D48">
-        <f t="shared" si="3"/>
-        <v>39</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F48">
+        <f t="shared" si="3"/>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="4"/>
       <c r="B49" t="s">
         <v>21</v>
       </c>
       <c r="C49">
+        <v>17</v>
+      </c>
+      <c r="D49">
+        <v>2</v>
+      </c>
+      <c r="E49">
         <f t="shared" si="2"/>
         <v>17</v>
       </c>
-      <c r="D49">
-        <f t="shared" si="3"/>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F49">
+        <f t="shared" si="3"/>
+        <v>63</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="4"/>
       <c r="B50" t="s">
         <v>22</v>
       </c>
       <c r="C50">
+        <v>17</v>
+      </c>
+      <c r="D50">
+        <v>4</v>
+      </c>
+      <c r="E50">
         <f t="shared" si="2"/>
         <v>18</v>
       </c>
-      <c r="D50">
-        <f t="shared" si="3"/>
-        <v>41</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F50">
+        <f t="shared" si="3"/>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="4"/>
       <c r="B51" t="s">
         <v>23</v>
       </c>
       <c r="C51">
+        <v>17</v>
+      </c>
+      <c r="D51">
+        <v>8</v>
+      </c>
+      <c r="E51">
         <f t="shared" si="2"/>
         <v>19</v>
       </c>
-      <c r="D51">
-        <f t="shared" si="3"/>
-        <v>42</v>
-      </c>
-    </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F51">
+        <f t="shared" si="3"/>
+        <v>65</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="4"/>
       <c r="B52" t="s">
         <v>24</v>
       </c>
       <c r="C52">
+        <v>17</v>
+      </c>
+      <c r="D52">
+        <v>10</v>
+      </c>
+      <c r="E52">
         <f t="shared" si="2"/>
         <v>20</v>
       </c>
-      <c r="D52">
-        <f t="shared" si="3"/>
-        <v>43</v>
-      </c>
-    </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F52">
+        <f t="shared" si="3"/>
+        <v>66</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="4"/>
       <c r="B53" t="s">
         <v>24</v>
       </c>
       <c r="C53">
+        <v>17</v>
+      </c>
+      <c r="D53">
+        <v>20</v>
+      </c>
+      <c r="E53">
         <f t="shared" si="2"/>
         <v>21</v>
       </c>
-      <c r="D53">
-        <f t="shared" si="3"/>
-        <v>44</v>
-      </c>
-    </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F53">
+        <f t="shared" si="3"/>
+        <v>67</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="4"/>
       <c r="B54" t="s">
         <v>24</v>
       </c>
       <c r="C54">
+        <v>17</v>
+      </c>
+      <c r="D54">
+        <v>40</v>
+      </c>
+      <c r="E54">
         <f t="shared" si="2"/>
         <v>22</v>
       </c>
-      <c r="D54">
-        <f t="shared" si="3"/>
-        <v>45</v>
-      </c>
-    </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F54">
+        <f t="shared" si="3"/>
+        <v>68</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="4"/>
       <c r="B55" t="s">
         <v>25</v>
       </c>
       <c r="C55">
+        <v>17</v>
+      </c>
+      <c r="D55">
+        <v>80</v>
+      </c>
+      <c r="E55">
         <f t="shared" si="2"/>
         <v>23</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="4"/>
       <c r="B56" t="s">
         <v>25</v>
       </c>
       <c r="C56">
+        <v>16</v>
+      </c>
+      <c r="D56">
+        <v>1</v>
+      </c>
+      <c r="E56">
         <f t="shared" si="2"/>
         <v>24</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="4"/>
       <c r="B57" t="s">
         <v>25</v>
       </c>
       <c r="C57">
+        <v>16</v>
+      </c>
+      <c r="D57">
+        <v>2</v>
+      </c>
+      <c r="E57">
         <f t="shared" si="2"/>
         <v>25</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="4"/>
       <c r="B58" t="s">
         <v>25</v>
       </c>
       <c r="C58">
+        <v>16</v>
+      </c>
+      <c r="D58">
+        <v>4</v>
+      </c>
+      <c r="E58">
         <f t="shared" si="2"/>
         <v>26</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="4"/>
       <c r="B59" t="s">
         <v>25</v>
       </c>
       <c r="C59">
+        <v>16</v>
+      </c>
+      <c r="D59">
+        <v>8</v>
+      </c>
+      <c r="E59">
         <f t="shared" si="2"/>
         <v>27</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="4"/>
       <c r="B60" t="s">
         <v>25</v>
       </c>
       <c r="C60">
+        <v>16</v>
+      </c>
+      <c r="D60">
+        <v>10</v>
+      </c>
+      <c r="E60">
         <f t="shared" si="2"/>
         <v>28</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="4"/>
       <c r="B61" t="s">
         <v>25</v>
       </c>
       <c r="C61">
-        <f>C60+1</f>
+        <v>16</v>
+      </c>
+      <c r="D61">
+        <v>20</v>
+      </c>
+      <c r="E61">
+        <f>E60+1</f>
         <v>29</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
-        <v>27</v>
+        <v>115</v>
       </c>
       <c r="B62" t="s">
         <v>4</v>
       </c>
       <c r="C62">
+        <v>30</v>
+      </c>
+      <c r="D62">
+        <v>1</v>
+      </c>
+      <c r="E62">
         <v>0</v>
       </c>
-      <c r="D62">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F62">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="4"/>
       <c r="B63" t="s">
         <v>5</v>
       </c>
       <c r="C63">
-        <f>C62+1</f>
+        <v>30</v>
+      </c>
+      <c r="D63">
+        <v>2</v>
+      </c>
+      <c r="E63">
+        <f>E62+1</f>
         <v>1</v>
       </c>
-      <c r="D63">
-        <f>D62+1</f>
-        <v>47</v>
-      </c>
-    </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F63">
+        <f>F62+1</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="4"/>
       <c r="B64" t="s">
         <v>6</v>
       </c>
       <c r="C64">
-        <f t="shared" ref="C64:C90" si="4">C63+1</f>
+        <v>30</v>
+      </c>
+      <c r="D64">
+        <v>4</v>
+      </c>
+      <c r="E64">
+        <f t="shared" ref="E64:E90" si="4">E63+1</f>
         <v>2</v>
       </c>
-      <c r="D64">
-        <f t="shared" ref="D64:D84" si="5">D63+1</f>
-        <v>48</v>
-      </c>
-    </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="F64">
+        <f t="shared" ref="F64:F84" si="5">F63+1</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="4"/>
       <c r="B65" t="s">
         <v>7</v>
       </c>
       <c r="C65">
+        <v>30</v>
+      </c>
+      <c r="D65">
+        <v>8</v>
+      </c>
+      <c r="E65">
         <f t="shared" si="4"/>
         <v>3</v>
       </c>
-      <c r="D65">
+      <c r="F65">
         <f t="shared" si="5"/>
-        <v>49</v>
-      </c>
-    </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.3">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="4"/>
       <c r="B66" t="s">
         <v>8</v>
       </c>
       <c r="C66">
+        <v>30</v>
+      </c>
+      <c r="D66">
+        <v>10</v>
+      </c>
+      <c r="E66">
         <f t="shared" si="4"/>
         <v>4</v>
       </c>
-      <c r="D66">
+      <c r="F66">
         <f t="shared" si="5"/>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.3">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="4"/>
       <c r="B67" t="s">
-        <v>9</v>
+        <v>23</v>
       </c>
       <c r="C67">
+        <v>30</v>
+      </c>
+      <c r="D67">
+        <v>20</v>
+      </c>
+      <c r="E67">
         <f t="shared" si="4"/>
         <v>5</v>
       </c>
-      <c r="D67">
+      <c r="F67">
         <f t="shared" si="5"/>
-        <v>51</v>
-      </c>
-    </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="4"/>
       <c r="B68" t="s">
-        <v>10</v>
+        <v>22</v>
       </c>
       <c r="C68">
+        <v>30</v>
+      </c>
+      <c r="D68">
+        <v>40</v>
+      </c>
+      <c r="E68">
         <f t="shared" si="4"/>
         <v>6</v>
       </c>
-      <c r="D68">
+      <c r="F68">
         <f t="shared" si="5"/>
-        <v>52</v>
-      </c>
-    </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="4"/>
       <c r="B69" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="C69">
+        <v>30</v>
+      </c>
+      <c r="D69">
+        <v>80</v>
+      </c>
+      <c r="E69">
         <f t="shared" si="4"/>
         <v>7</v>
       </c>
-      <c r="D69">
+      <c r="F69">
         <f t="shared" si="5"/>
-        <v>53</v>
-      </c>
-    </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.3">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="4"/>
       <c r="B70" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="C70">
-        <f t="shared" si="4"/>
-        <v>8</v>
+        <v>29</v>
       </c>
       <c r="D70">
+        <v>1</v>
+      </c>
+      <c r="E70">
+        <f t="shared" si="4"/>
+        <v>8</v>
+      </c>
+      <c r="F70">
         <f t="shared" si="5"/>
-        <v>54</v>
-      </c>
-    </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="4"/>
       <c r="B71" t="s">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="C71">
+        <v>29</v>
+      </c>
+      <c r="D71">
+        <v>2</v>
+      </c>
+      <c r="E71">
         <f t="shared" si="4"/>
         <v>9</v>
       </c>
-      <c r="D71">
+      <c r="F71">
         <f t="shared" si="5"/>
-        <v>55</v>
-      </c>
-    </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.3">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="4"/>
       <c r="B72" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="C72">
+        <v>29</v>
+      </c>
+      <c r="D72">
+        <v>4</v>
+      </c>
+      <c r="E72">
         <f t="shared" si="4"/>
         <v>10</v>
       </c>
-      <c r="D72">
+      <c r="F72">
         <f t="shared" si="5"/>
-        <v>56</v>
-      </c>
-    </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.3">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="4"/>
       <c r="B73" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C73">
+        <v>29</v>
+      </c>
+      <c r="D73">
+        <v>8</v>
+      </c>
+      <c r="E73">
         <f t="shared" si="4"/>
         <v>11</v>
       </c>
-      <c r="D73">
+      <c r="F73">
         <f t="shared" si="5"/>
-        <v>57</v>
-      </c>
-    </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="4"/>
       <c r="B74" t="s">
         <v>16</v>
       </c>
       <c r="C74">
+        <v>29</v>
+      </c>
+      <c r="D74">
+        <v>10</v>
+      </c>
+      <c r="E74">
         <f t="shared" si="4"/>
         <v>12</v>
       </c>
-      <c r="D74">
+      <c r="F74">
         <f t="shared" si="5"/>
-        <v>58</v>
-      </c>
-    </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.3">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="4"/>
       <c r="B75" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C75">
+        <v>29</v>
+      </c>
+      <c r="D75">
+        <v>20</v>
+      </c>
+      <c r="E75">
         <f t="shared" si="4"/>
         <v>13</v>
       </c>
-      <c r="D75">
+      <c r="F75">
         <f t="shared" si="5"/>
-        <v>59</v>
-      </c>
-    </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.3">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="4"/>
       <c r="B76" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C76">
+        <v>29</v>
+      </c>
+      <c r="D76">
+        <v>40</v>
+      </c>
+      <c r="E76">
         <f t="shared" si="4"/>
         <v>14</v>
       </c>
-      <c r="D76">
+      <c r="F76">
         <f t="shared" si="5"/>
-        <v>60</v>
-      </c>
-    </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.3">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="4"/>
       <c r="B77" t="s">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="C77">
+        <v>29</v>
+      </c>
+      <c r="D77">
+        <v>80</v>
+      </c>
+      <c r="E77">
         <f t="shared" si="4"/>
         <v>15</v>
       </c>
-      <c r="D77">
+      <c r="F77">
         <f t="shared" si="5"/>
-        <v>61</v>
-      </c>
-    </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="4"/>
       <c r="B78" t="s">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="C78">
+        <v>28</v>
+      </c>
+      <c r="D78">
+        <v>1</v>
+      </c>
+      <c r="E78">
         <f t="shared" si="4"/>
         <v>16</v>
       </c>
-      <c r="D78">
+      <c r="F78">
         <f t="shared" si="5"/>
-        <v>62</v>
-      </c>
-    </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.3">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="4"/>
       <c r="B79" t="s">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="C79">
+        <v>28</v>
+      </c>
+      <c r="D79">
+        <v>2</v>
+      </c>
+      <c r="E79">
         <f t="shared" si="4"/>
         <v>17</v>
       </c>
-      <c r="D79">
+      <c r="F79">
         <f t="shared" si="5"/>
-        <v>63</v>
-      </c>
-    </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.3">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="4"/>
       <c r="B80" t="s">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="C80">
+        <v>28</v>
+      </c>
+      <c r="D80">
+        <v>4</v>
+      </c>
+      <c r="E80">
         <f t="shared" si="4"/>
         <v>18</v>
       </c>
-      <c r="D80">
+      <c r="F80">
         <f t="shared" si="5"/>
-        <v>64</v>
-      </c>
-    </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.3">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="4"/>
       <c r="B81" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="C81">
+        <v>28</v>
+      </c>
+      <c r="D81">
+        <v>8</v>
+      </c>
+      <c r="E81">
         <f t="shared" si="4"/>
         <v>19</v>
       </c>
-      <c r="D81">
+      <c r="F81">
         <f t="shared" si="5"/>
-        <v>65</v>
-      </c>
-    </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.3">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="4"/>
       <c r="B82" t="s">
         <v>24</v>
       </c>
       <c r="C82">
+        <v>28</v>
+      </c>
+      <c r="D82">
+        <v>10</v>
+      </c>
+      <c r="E82">
         <f t="shared" si="4"/>
         <v>20</v>
       </c>
-      <c r="D82">
+      <c r="F82">
         <f t="shared" si="5"/>
-        <v>66</v>
-      </c>
-    </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.3">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="4"/>
       <c r="B83" t="s">
         <v>24</v>
       </c>
       <c r="C83">
+        <v>28</v>
+      </c>
+      <c r="D83">
+        <v>20</v>
+      </c>
+      <c r="E83">
         <f t="shared" si="4"/>
         <v>21</v>
       </c>
-      <c r="D83">
+      <c r="F83">
         <f t="shared" si="5"/>
-        <v>67</v>
-      </c>
-    </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.3">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="4"/>
       <c r="B84" t="s">
         <v>24</v>
       </c>
       <c r="C84">
+        <v>28</v>
+      </c>
+      <c r="D84">
+        <v>40</v>
+      </c>
+      <c r="E84">
         <f t="shared" si="4"/>
         <v>22</v>
       </c>
-      <c r="D84">
+      <c r="F84">
         <f t="shared" si="5"/>
-        <v>68</v>
-      </c>
-    </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.3">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="4"/>
       <c r="B85" t="s">
         <v>25</v>
       </c>
       <c r="C85">
+        <v>28</v>
+      </c>
+      <c r="D85">
+        <v>80</v>
+      </c>
+      <c r="E85">
         <f t="shared" si="4"/>
         <v>23</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="4"/>
       <c r="B86" t="s">
         <v>25</v>
       </c>
       <c r="C86">
+        <v>27</v>
+      </c>
+      <c r="D86">
+        <v>1</v>
+      </c>
+      <c r="E86">
         <f t="shared" si="4"/>
         <v>24</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="4"/>
       <c r="B87" t="s">
         <v>25</v>
       </c>
       <c r="C87">
+        <v>27</v>
+      </c>
+      <c r="D87">
+        <v>2</v>
+      </c>
+      <c r="E87">
         <f t="shared" si="4"/>
         <v>25</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="4"/>
       <c r="B88" t="s">
         <v>25</v>
       </c>
       <c r="C88">
+        <v>27</v>
+      </c>
+      <c r="D88">
+        <v>4</v>
+      </c>
+      <c r="E88">
         <f t="shared" si="4"/>
         <v>26</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="4"/>
       <c r="B89" t="s">
         <v>25</v>
       </c>
       <c r="C89">
-        <f t="shared" si="4"/>
         <v>27</v>
       </c>
-    </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="D89">
+        <v>8</v>
+      </c>
+      <c r="E89">
+        <f t="shared" si="4"/>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="4"/>
       <c r="B90" t="s">
         <v>25</v>
       </c>
       <c r="C90">
+        <v>27</v>
+      </c>
+      <c r="D90">
+        <v>10</v>
+      </c>
+      <c r="E90">
         <f t="shared" si="4"/>
         <v>28</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="4"/>
       <c r="B91" t="s">
         <v>25</v>
       </c>
       <c r="C91">
-        <f>C90+1</f>
+        <v>27</v>
+      </c>
+      <c r="D91">
+        <v>20</v>
+      </c>
+      <c r="E91">
+        <f>E90+1</f>
         <v>29</v>
       </c>
+    </row>
+    <row r="97" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C97" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="98" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C98" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="99" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C99" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="100" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C100" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="101" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C101" s="2" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="102" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C102" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="106" spans="3:4" x14ac:dyDescent="0.3">
+      <c r="C106" s="3"/>
+      <c r="D106" s="3"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>